<commit_message>
Daily EOD data and reports for 2026-10-12
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20261012.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20261012.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.767</v>
+        <v>1.775</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.003</v>
+        <v>0.005</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.17%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>270670.83</v>
+        <v>271896.27</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-459.54</v>
+        <v>765.9</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.43</v>
+        <v>2.44</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.41%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>170100</v>
+        <v>170800</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>62.27</v>
+        <v>62.46</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>1.33</v>
+        <v>1.52</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2.18%</t>
+          <t>2.49%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>498160</v>
+        <v>499680</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>10640</v>
+        <v>12160</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0</v>
+        <v>0.006</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.006</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0</v>
+        <v>264.54</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-264.54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>148.89</v>
+        <v>149.46</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-0.4</v>
+        <v>0.17</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-0.27%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.885</v>
+        <v>0.89</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.72%</t>
+          <t>2.30%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>8850</v>
+        <v>8900</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>184.16</v>
+        <v>184.02</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.32</v>
+        <v>0.18</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>0.10%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>736640</v>
+        <v>736080</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>1280</v>
+        <v>720</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.245</v>
+        <v>-0.005</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-2.04%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0</v>
+        <v>4800</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-4900</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="12">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.097</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.098</v>
+        <v>-0.001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-1.02%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>582</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-588</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>33.94</v>
+        <v>34.09</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.22</v>
+        <v>0.37</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>1.10%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.1</v>
+        <v>31.98</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.22</v>
+        <v>-0.34</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-0.68%</t>
+          <t>-1.05%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>41344.8</v>
+        <v>41190.24</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-283.36</v>
+        <v>-437.92</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1769804.65</v>
+        <v>1778232.07</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>3706.53</v>
+        <v>12133.96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>